<commit_message>
Fix narrative assembly bindings, interaction priority and Trials keyboard focus
</commit_message>
<xml_diff>
--- a/docs/forge/xeno-trials/XENO_TRIALS_SUIVI_V156.xlsx
+++ b/docs/forge/xeno-trials/XENO_TRIALS_SUIVI_V156.xlsx
@@ -1309,7 +1309,7 @@
       </c>
       <c r="F7" s="1" t="inlineStr">
         <is>
-          <t>Réponse à la famille effective de l’adversaire pendant sa présentation ; aucune rivalité historique affirmée. Adaptation de simulation ; dessins complets, audio et relevés d’œuvre restent ouverts. Aucun lot artistique clos ni certification 1:1.</t>
+          <t>Réponse à la famille effective de l’adversaire, y compris hybride, pendant sa présentation ; aucune rivalité historique affirmée. Adaptation de simulation ; dessins complets, audio et relevés d’œuvre restent ouverts. Aucun lot artistique clos ni certification 1:1.</t>
         </is>
       </c>
       <c r="G7" s="1" t="n">
@@ -1575,7 +1575,7 @@
       </c>
       <c r="F14" s="1" t="inlineStr">
         <is>
-          <t>Commande T ou bouton dédié pendant le combat ; annulation par déplacement, attaque, garde ou impact. Adaptation de simulation ; dessins complets, audio et relevés d’œuvre restent ouverts. Aucun lot artistique clos ni certification 1:1.</t>
+          <t>Commande T ou bouton DÉFI pendant le combat ; le bouton rend le focus au canvas quand le combat accepte les commandes. Annulation par déplacement, attaque, garde ou impact. Adaptation de simulation ; dessins complets, audio et relevés d’œuvre restent ouverts. Aucun lot artistique clos ni certification 1:1.</t>
         </is>
       </c>
       <c r="G14" s="1" t="n">
@@ -1689,7 +1689,7 @@
       </c>
       <c r="F17" s="1" t="inlineStr">
         <is>
-          <t>Réponse à la famille effective de l’adversaire pendant sa présentation ; aucune rivalité historique affirmée. Adaptation de simulation ; dessins complets, audio et relevés d’œuvre restent ouverts. Aucun lot artistique clos ni certification 1:1.</t>
+          <t>Réponse à la famille effective de l’adversaire, y compris hybride, pendant sa présentation ; aucune rivalité historique affirmée. Adaptation de simulation ; dessins complets, audio et relevés d’œuvre restent ouverts. Aucun lot artistique clos ni certification 1:1.</t>
         </is>
       </c>
       <c r="G17" s="1" t="n">
@@ -1955,7 +1955,7 @@
       </c>
       <c r="F24" s="1" t="inlineStr">
         <is>
-          <t>Commande T ou bouton dédié pendant le combat ; annulation par déplacement, attaque, garde ou impact. Adaptation de simulation ; dessins complets, audio et relevés d’œuvre restent ouverts. Aucun lot artistique clos ni certification 1:1.</t>
+          <t>Commande T ou bouton DÉFI pendant le combat ; le bouton rend le focus au canvas quand le combat accepte les commandes. Annulation par déplacement, attaque, garde ou impact. Adaptation de simulation ; dessins complets, audio et relevés d’œuvre restent ouverts. Aucun lot artistique clos ni certification 1:1.</t>
         </is>
       </c>
       <c r="G24" s="1" t="n">
@@ -2069,7 +2069,7 @@
       </c>
       <c r="F27" s="1" t="inlineStr">
         <is>
-          <t>Réponse à la famille effective de l’adversaire pendant sa présentation ; aucune rivalité historique affirmée. Adaptation de simulation ; dessins complets, audio et relevés d’œuvre restent ouverts. Aucun lot artistique clos ni certification 1:1.</t>
+          <t>Réponse à la famille effective de l’adversaire, y compris hybride, pendant sa présentation ; aucune rivalité historique affirmée. Adaptation de simulation ; dessins complets, audio et relevés d’œuvre restent ouverts. Aucun lot artistique clos ni certification 1:1.</t>
         </is>
       </c>
       <c r="G27" s="1" t="n">
@@ -2335,7 +2335,7 @@
       </c>
       <c r="F34" s="1" t="inlineStr">
         <is>
-          <t>Commande T ou bouton dédié pendant le combat ; annulation par déplacement, attaque, garde ou impact. Adaptation de simulation ; dessins complets, audio et relevés d’œuvre restent ouverts. Aucun lot artistique clos ni certification 1:1.</t>
+          <t>Commande T ou bouton DÉFI pendant le combat ; le bouton rend le focus au canvas quand le combat accepte les commandes. Annulation par déplacement, attaque, garde ou impact. Adaptation de simulation ; dessins complets, audio et relevés d’œuvre restent ouverts. Aucun lot artistique clos ni certification 1:1.</t>
         </is>
       </c>
       <c r="G34" s="1" t="n">
@@ -2449,7 +2449,7 @@
       </c>
       <c r="F37" s="1" t="inlineStr">
         <is>
-          <t>Réponse à la famille effective de l’adversaire pendant sa présentation ; aucune rivalité historique affirmée. Adaptation de simulation ; dessins complets, audio et relevés d’œuvre restent ouverts. Aucun lot artistique clos ni certification 1:1.</t>
+          <t>Réponse à la famille effective de l’adversaire, y compris hybride, pendant sa présentation ; aucune rivalité historique affirmée. Adaptation de simulation ; dessins complets, audio et relevés d’œuvre restent ouverts. Aucun lot artistique clos ni certification 1:1.</t>
         </is>
       </c>
       <c r="G37" s="1" t="n">
@@ -2715,7 +2715,7 @@
       </c>
       <c r="F44" s="1" t="inlineStr">
         <is>
-          <t>Commande T ou bouton dédié pendant le combat ; annulation par déplacement, attaque, garde ou impact. Adaptation de simulation ; dessins complets, audio et relevés d’œuvre restent ouverts. Aucun lot artistique clos ni certification 1:1.</t>
+          <t>Commande T ou bouton DÉFI pendant le combat ; le bouton rend le focus au canvas quand le combat accepte les commandes. Annulation par déplacement, attaque, garde ou impact. Adaptation de simulation ; dessins complets, audio et relevés d’œuvre restent ouverts. Aucun lot artistique clos ni certification 1:1.</t>
         </is>
       </c>
       <c r="G44" s="1" t="n">
@@ -6570,7 +6570,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="39" customWidth="1" min="2" max="2"/>
     <col width="40" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="40" customWidth="1" min="5" max="5"/>
@@ -6782,12 +6782,12 @@
       </c>
       <c r="B11" s="1" t="inlineStr">
         <is>
-          <t>Édition et conservation du document</t>
+          <t>Édition, assemblages et versionnement</t>
         </is>
       </c>
       <c r="C11" s="1" t="inlineStr">
         <is>
-          <t>Inspecteur natif, annuler/rétablir, JSON schema3, versions V136 et différences</t>
+          <t>Inspecteur, annuler/rétablir, JSON schema 3 et versions V136 ; capture, bibliothèque, rotation et pose préservent les références aux objectifs externes.</t>
         </is>
       </c>
       <c r="D11" s="1" t="inlineStr">
@@ -6797,7 +6797,7 @@
       </c>
       <c r="E11" s="1" t="inlineStr">
         <is>
-          <t>Le versionnement concerne le document, pas la progression d’une partie.</t>
+          <t>La validation du projet reste stricte. L’aperçu et la pose refusent les références absentes, décoratives ou en conflit physique.</t>
         </is>
       </c>
     </row>
@@ -6814,7 +6814,7 @@
       </c>
       <c r="C12" s="1" t="inlineStr">
         <is>
-          <t>Terminal réel, E, fenêtre DOM clavier/clic ; monde suspendu</t>
+          <t>Terminal réel le plus proche, E, fenêtre DOM clavier/clic et monde suspendu ; un objectif plus proche physiquement activable reste prioritaire.</t>
         </is>
       </c>
       <c r="D12" s="1" t="inlineStr">

</xml_diff>

<commit_message>
Preserve native interaction admission and recovery priorities in Forge
</commit_message>
<xml_diff>
--- a/docs/forge/xeno-trials/XENO_TRIALS_SUIVI_V156.xlsx
+++ b/docs/forge/xeno-trials/XENO_TRIALS_SUIVI_V156.xlsx
@@ -6814,7 +6814,7 @@
       </c>
       <c r="C12" s="1" t="inlineStr">
         <is>
-          <t>Terminal réel le plus proche, E, fenêtre DOM clavier/clic et monde suspendu ; un objectif plus proche physiquement activable reste prioritaire.</t>
+          <t>E choisit une action admissible : récit, terminal ordinaire encore à activer ou objectif prêt. Verrou boss et prompts natifs conservés ; réanimation J2, clé et récupération d’arme déléguées au moteur natif.</t>
         </is>
       </c>
       <c r="D12" s="1" t="inlineStr">
@@ -6824,7 +6824,7 @@
       </c>
       <c r="E12" s="1" t="inlineStr">
         <is>
-          <t>Les scénarios navigateur et contrôle du commit exact sont vérifiés séparément.</t>
+          <t>Monde suspendu pendant le récit ; sans nouveau gain ni affaiblissement des prérequis. Récupération Bow/Harpoon : profil équipé, propriétaire, portée 72 et ligne de vue native conservés.</t>
         </is>
       </c>
     </row>
@@ -7277,7 +7277,7 @@
       </c>
       <c r="B10" s="1" t="inlineStr">
         <is>
-          <t>node --test scripts/verify-forge-narrative-v156.mjs</t>
+          <t>node --test scripts/verify-forge-narrative-v156.mjs scripts/verify-weapon-actions-v131.mjs</t>
         </is>
       </c>
       <c r="C10" s="1" t="inlineStr">
@@ -7287,7 +7287,7 @@
       </c>
       <c r="D10" s="1" t="inlineStr">
         <is>
-          <t>Projet, inspecteur, branches, objectifs, sessions et moteurs natifs.</t>
+          <t>Projets, assemblages, choix, priorités natives et récupération Bow/Harpoon ; aucune CI anticipée.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Gate native Forge delegation and preserve objective confirmation
</commit_message>
<xml_diff>
--- a/docs/forge/xeno-trials/XENO_TRIALS_SUIVI_V156.xlsx
+++ b/docs/forge/xeno-trials/XENO_TRIALS_SUIVI_V156.xlsx
@@ -6814,7 +6814,7 @@
       </c>
       <c r="C12" s="1" t="inlineStr">
         <is>
-          <t>E choisit une action admissible : récit, terminal ordinaire encore à activer ou objectif prêt. Verrou boss et prompts natifs conservés ; réanimation J2, clé et récupération d’arme déléguées au moteur natif.</t>
+          <t>E choisit une action admissible ; admission commune aux actions et prompts natifs power/archive. Ordre power→archive après visibilité et verrou boss. Réanimation J2, clé et récupération restent déléguées au moteur natif.</t>
         </is>
       </c>
       <c r="D12" s="1" t="inlineStr">
@@ -6824,7 +6824,7 @@
       </c>
       <c r="E12" s="1" t="inlineStr">
         <is>
-          <t>Monde suspendu pendant le récit ; sans nouveau gain ni affaiblissement des prérequis. Récupération Bow/Harpoon : profil équipé, propriétaire, portée 72 et ligne de vue native conservés.</t>
+          <t>Récupération seulement sans terminal en attente admis, sans objectif proche ni porte native cloisonnée ; profil, propriétaire, portée 72 et ligne de vue natifs conservés. Hors Forge : conditions historiques inchangées.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Stop controller action batches when a Forge story opens
</commit_message>
<xml_diff>
--- a/docs/forge/xeno-trials/XENO_TRIALS_SUIVI_V156.xlsx
+++ b/docs/forge/xeno-trials/XENO_TRIALS_SUIVI_V156.xlsx
@@ -6814,7 +6814,7 @@
       </c>
       <c r="C12" s="1" t="inlineStr">
         <is>
-          <t>E choisit une action admissible ; admission commune aux actions et prompts natifs power/archive. Ordre power→archive après visibilité et verrou boss. Réanimation J2, clé et récupération restent déléguées au moteur natif.</t>
+          <t>E choisit une action admissible ; admission commune aux actions et prompts natifs power/archive. Ordre power→archive après visibilité et verrou boss. Réanimation J2, clé et récupération restent déléguées au moteur natif. À la manette, admission avant les actions et arrêt du lot dès l’ouverture d’un récit, pour les deux joueurs.</t>
         </is>
       </c>
       <c r="D12" s="1" t="inlineStr">
@@ -6824,7 +6824,7 @@
       </c>
       <c r="E12" s="1" t="inlineStr">
         <is>
-          <t>Récupération seulement sans terminal en attente admis, sans objectif proche ni porte native cloisonnée ; profil, propriétaire, portée 72 et ligne de vue natifs conservés. Hors Forge : conditions historiques inchangées.</t>
+          <t>Récupération seulement sans terminal en attente admis, sans objectif proche ni porte native cloisonnée ; profil, propriétaire, portée 72 et ligne de vue natifs conservés. Hors Forge : conditions historiques inchangées. Réarmement au neutre ; le refus direct du véhicule précède toute annulation de travail ou d’aperçu.</t>
         </is>
       </c>
     </row>

</xml_diff>